<commit_message>
bruto netto index verschillen er bij
</commit_message>
<xml_diff>
--- a/Actiam/Actiam-KostenBepaling2020.xlsx
+++ b/Actiam/Actiam-KostenBepaling2020.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GoogleDrive\Financieel\Aandelen\KeuzeWelkIndexFonds\PerFonds\Actiam\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB87FF82-FE1D-45C3-83BB-57921F1D0578}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21449A73-3CF6-414A-A6DD-6F9BA867FAF6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -89,7 +89,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B15" authorId="0" shapeId="0" xr:uid="{9B32E177-9E47-4B8A-BA3D-C6E6BC6434F4}">
+    <comment ref="B18" authorId="0" shapeId="0" xr:uid="{9B32E177-9E47-4B8A-BA3D-C6E6BC6434F4}">
       <text>
         <r>
           <rPr>
@@ -119,7 +119,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="39">
   <si>
     <t>Gemiddelde</t>
   </si>
@@ -230,18 +230,25 @@
   </si>
   <si>
     <t>ESG verchil volgens jaarverslag tov volledige index</t>
+  </si>
+  <si>
+    <t>Bruto netto index verschil</t>
+  </si>
+  <si>
+    <t>gemiddeld bruto netto index verschil</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="44" formatCode="_ &quot;€&quot;\ * #,##0.00_ ;_ &quot;€&quot;\ * \-#,##0.00_ ;_ &quot;€&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="164" formatCode="_ &quot;€&quot;\ * #,##0_ ;_ &quot;€&quot;\ * \-#,##0_ ;_ &quot;€&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="165" formatCode="0.000%"/>
-    <numFmt numFmtId="168" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="0.000"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
@@ -368,7 +375,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -391,7 +398,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="3" applyFont="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1"/>
@@ -406,8 +413,9 @@
     </xf>
     <xf numFmtId="2" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Komma" xfId="3" builtinId="3"/>
@@ -426,10 +434,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1110,13 +1114,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F528616F-4365-4E03-AA99-F5C2282C78C2}">
-  <dimension ref="B1:J22"/>
+  <dimension ref="B1:K25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="C1" s="14">
         <v>2016</v>
       </c>
@@ -1137,7 +1141,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2" s="15" t="s">
         <v>23</v>
       </c>
@@ -1157,7 +1161,7 @@
       <c r="H2" s="13"/>
       <c r="I2" s="13"/>
     </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="15" t="s">
         <v>32</v>
       </c>
@@ -1177,7 +1181,7 @@
       <c r="H3" s="13"/>
       <c r="I3" s="13"/>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B4" s="15" t="s">
         <v>33</v>
       </c>
@@ -1197,7 +1201,7 @@
       <c r="H4" s="13"/>
       <c r="I4" s="13"/>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" s="15" t="s">
         <v>9</v>
       </c>
@@ -1224,7 +1228,7 @@
         <v>0.42999999999999994</v>
       </c>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" s="15" t="s">
         <v>8</v>
       </c>
@@ -1251,272 +1255,335 @@
       </c>
       <c r="I6" s="13"/>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B7" s="15"/>
-      <c r="C7" s="28"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="28"/>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B7" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="28">
+        <f>C3-C4</f>
+        <v>0.66000000000000014</v>
+      </c>
+      <c r="D7" s="28">
+        <f t="shared" ref="D7:F7" si="0">D3-D4</f>
+        <v>0.58999999999999986</v>
+      </c>
+      <c r="E7" s="28">
+        <f t="shared" si="0"/>
+        <v>0.53000000000000025</v>
+      </c>
+      <c r="F7" s="28">
+        <f t="shared" si="0"/>
+        <v>0.65000000000000213</v>
+      </c>
       <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="16"/>
-    </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B8" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="C8" s="28">
-        <v>0.03</v>
-      </c>
-      <c r="D8" s="28">
-        <v>-0.1</v>
-      </c>
-      <c r="E8" s="28">
-        <v>0.31</v>
-      </c>
-      <c r="F8" s="28">
-        <v>-0.17</v>
-      </c>
+      <c r="H7" s="16"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="32">
+        <f>AVERAGE(C7:F7)</f>
+        <v>0.6075000000000006</v>
+      </c>
+      <c r="K7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B8" s="15"/>
+      <c r="C8" s="28"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="28"/>
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
-      <c r="I8" s="13"/>
-    </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="I8" s="16"/>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B9" s="15" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="C9" s="28">
-        <f>C5-C8</f>
-        <v>0.55000000000000004</v>
+        <v>0.03</v>
       </c>
       <c r="D9" s="28">
-        <f>D5-D8</f>
-        <v>0.26999999999999991</v>
+        <v>-0.1</v>
       </c>
       <c r="E9" s="28">
-        <f>E5-E8</f>
-        <v>0.21000000000000046</v>
+        <v>0.31</v>
       </c>
       <c r="F9" s="28">
-        <f>F5-F8</f>
-        <v>0.61999999999999933</v>
+        <v>-0.17</v>
       </c>
       <c r="G9" s="13"/>
       <c r="H9" s="13"/>
-      <c r="I9" s="16">
-        <f>AVERAGE(C9:F9)</f>
+      <c r="I9" s="13"/>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B10" s="15"/>
+      <c r="C10" s="28">
+        <f>C2-C9</f>
+        <v>11.280000000000001</v>
+      </c>
+      <c r="D10" s="28">
+        <f t="shared" ref="D10:F10" si="1">D2-D9</f>
+        <v>7.7799999999999994</v>
+      </c>
+      <c r="E10" s="28">
+        <f t="shared" si="1"/>
+        <v>-3.9</v>
+      </c>
+      <c r="F10" s="28">
+        <f t="shared" si="1"/>
+        <v>30.64</v>
+      </c>
+      <c r="G10" s="13"/>
+      <c r="H10" s="13"/>
+      <c r="I10" s="13"/>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B11" s="15"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="13"/>
+      <c r="I11" s="13"/>
+    </row>
+    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B12" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="28">
+        <f>C5-C9</f>
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="D12" s="28">
+        <f>D5-D9</f>
+        <v>0.26999999999999991</v>
+      </c>
+      <c r="E12" s="28">
+        <f>E5-E9</f>
+        <v>0.21000000000000046</v>
+      </c>
+      <c r="F12" s="28">
+        <f>F5-F9</f>
+        <v>0.61999999999999933</v>
+      </c>
+      <c r="G12" s="13"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="16">
+        <f>AVERAGE(C12:F12)</f>
         <v>0.41249999999999998</v>
       </c>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B10" s="15" t="s">
+    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B13" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="28">
-        <f>C6+C8</f>
+      <c r="C13" s="28">
+        <f>C6+C9</f>
         <v>0.11000000000000007</v>
       </c>
-      <c r="D10" s="28">
-        <f>D6+D8</f>
+      <c r="D13" s="28">
+        <f>D6+D9</f>
         <v>0.31999999999999995</v>
       </c>
-      <c r="E10" s="28">
-        <f>E6+E8</f>
+      <c r="E13" s="28">
+        <f>E6+E9</f>
         <v>0.31999999999999978</v>
       </c>
-      <c r="F10" s="28">
-        <f>F6+F8</f>
+      <c r="F13" s="28">
+        <f>F6+F9</f>
         <v>3.000000000000283E-2</v>
       </c>
-      <c r="G10" s="13"/>
-      <c r="H10" s="31">
-        <f>AVERAGE(C10:F10)</f>
+      <c r="G13" s="13"/>
+      <c r="H13" s="33">
+        <f>AVERAGE(C13:F13)</f>
         <v>0.19500000000000065</v>
       </c>
-      <c r="I10" s="13"/>
-    </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B13" s="30" t="s">
+      <c r="I13" s="13"/>
+    </row>
+    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B16" s="30" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B14" s="18" t="s">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B17" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="D14" s="29">
+      <c r="D17" s="29">
         <v>8.02</v>
       </c>
-      <c r="E14" s="19">
+      <c r="E17" s="19">
         <v>-10.92</v>
       </c>
-      <c r="F14" s="17">
+      <c r="F17" s="17">
         <v>20.13</v>
       </c>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="19"/>
-      <c r="J14" s="17"/>
-    </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B15" s="18" t="s">
+      <c r="G17" s="17"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="19"/>
+      <c r="J17" s="17"/>
+    </row>
+    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B18" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="D15" s="29">
+      <c r="D18" s="29">
         <v>8.6</v>
       </c>
-      <c r="E15" s="19">
+      <c r="E18" s="19">
         <v>-9.91</v>
       </c>
-      <c r="F15" s="17">
+      <c r="F18" s="17">
         <v>21.07</v>
       </c>
-      <c r="G15" s="17"/>
-      <c r="H15" s="19"/>
-      <c r="I15" s="19"/>
-      <c r="J15" s="17"/>
-    </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B16" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="29">
-        <v>8.31</v>
-      </c>
-      <c r="E16" s="19">
-        <v>-10.26</v>
-      </c>
-      <c r="F16" s="17">
-        <v>20.6</v>
-      </c>
-      <c r="G16" s="17"/>
-      <c r="H16" s="19"/>
-      <c r="I16" s="19"/>
-      <c r="J16" s="17"/>
-    </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B17" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="D17" s="29">
-        <f>D14-D16</f>
-        <v>-0.29000000000000092</v>
-      </c>
-      <c r="E17" s="19">
-        <f>E14-E16</f>
-        <v>-0.66000000000000014</v>
-      </c>
-      <c r="F17" s="19">
-        <f>F14-F16</f>
-        <v>-0.47000000000000242</v>
-      </c>
-      <c r="G17" s="19"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="19">
-        <f>AVERAGE(D17:F17)</f>
-        <v>-0.47333333333333449</v>
-      </c>
-      <c r="J17" s="17"/>
-    </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B18" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="D18" s="29">
-        <f>D15-D14</f>
-        <v>0.58000000000000007</v>
-      </c>
-      <c r="E18" s="19">
-        <f>E15-E14</f>
-        <v>1.0099999999999998</v>
-      </c>
-      <c r="F18" s="19">
-        <f>F15-F14</f>
-        <v>0.94000000000000128</v>
-      </c>
-      <c r="G18" s="19"/>
-      <c r="H18" s="19">
-        <f>AVERAGE(D18:F18)</f>
-        <v>0.84333333333333371</v>
-      </c>
+      <c r="G18" s="17"/>
+      <c r="H18" s="19"/>
       <c r="I18" s="19"/>
       <c r="J18" s="17"/>
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B19" s="18"/>
-      <c r="D19" s="29"/>
-      <c r="E19" s="19"/>
-      <c r="F19" s="19"/>
-      <c r="G19" s="19"/>
+      <c r="B19" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="D19" s="29">
+        <v>8.31</v>
+      </c>
+      <c r="E19" s="19">
+        <v>-10.26</v>
+      </c>
+      <c r="F19" s="17">
+        <v>20.6</v>
+      </c>
+      <c r="G19" s="17"/>
       <c r="H19" s="19"/>
       <c r="I19" s="19"/>
       <c r="J19" s="17"/>
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B20" s="15" t="s">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="D20" s="29">
-        <v>0.43</v>
+        <f>D17-D19</f>
+        <v>-0.29000000000000092</v>
       </c>
       <c r="E20" s="19">
-        <v>-0.31</v>
-      </c>
-      <c r="F20" s="17">
-        <v>-7.0000000000000007E-2</v>
-      </c>
-      <c r="G20" s="17"/>
-      <c r="H20" s="17"/>
-      <c r="I20" s="19"/>
-      <c r="J20" s="19"/>
+        <f>E17-E19</f>
+        <v>-0.66000000000000014</v>
+      </c>
+      <c r="F20" s="19">
+        <f>F17-F19</f>
+        <v>-0.47000000000000242</v>
+      </c>
+      <c r="G20" s="19"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="19">
+        <f>AVERAGE(D20:F20)</f>
+        <v>-0.47333333333333449</v>
+      </c>
+      <c r="J20" s="17"/>
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B21" s="18" t="s">
-        <v>30</v>
+      <c r="B21" s="15" t="s">
+        <v>8</v>
       </c>
       <c r="D21" s="29">
-        <f>D17-D20</f>
-        <v>-0.72000000000000086</v>
+        <f>D18-D17</f>
+        <v>0.58000000000000007</v>
       </c>
       <c r="E21" s="19">
-        <f>E17-E20</f>
-        <v>-0.35000000000000014</v>
+        <f>E18-E17</f>
+        <v>1.0099999999999998</v>
       </c>
       <c r="F21" s="19">
-        <f>F17-F20</f>
-        <v>-0.40000000000000241</v>
-      </c>
-      <c r="G21" s="17"/>
-      <c r="H21" s="19"/>
-      <c r="I21" s="19">
+        <f>F18-F17</f>
+        <v>0.94000000000000128</v>
+      </c>
+      <c r="G21" s="19"/>
+      <c r="H21" s="19">
         <f>AVERAGE(D21:F21)</f>
-        <v>-0.4900000000000011</v>
-      </c>
+        <v>0.84333333333333371</v>
+      </c>
+      <c r="I21" s="19"/>
       <c r="J21" s="17"/>
     </row>
     <row r="22" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B22" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="D22" s="29">
-        <f>D18+D20</f>
-        <v>1.01</v>
-      </c>
-      <c r="E22" s="19">
-        <f>E18+E20</f>
-        <v>0.69999999999999973</v>
-      </c>
-      <c r="F22" s="19">
-        <f>F18+F20</f>
-        <v>0.87000000000000122</v>
-      </c>
-      <c r="G22" s="17"/>
-      <c r="H22" s="32">
-        <f>AVERAGE(D22:F22)</f>
-        <v>0.86000000000000032</v>
-      </c>
+      <c r="B22" s="18"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="19"/>
+      <c r="G22" s="19"/>
+      <c r="H22" s="19"/>
       <c r="I22" s="19"/>
       <c r="J22" s="17"/>
+    </row>
+    <row r="23" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B23" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="D23" s="29">
+        <v>0.43</v>
+      </c>
+      <c r="E23" s="19">
+        <v>-0.31</v>
+      </c>
+      <c r="F23" s="17">
+        <v>-7.0000000000000007E-2</v>
+      </c>
+      <c r="G23" s="17"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="19"/>
+      <c r="J23" s="19"/>
+    </row>
+    <row r="24" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B24" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="D24" s="29">
+        <f>D20-D23</f>
+        <v>-0.72000000000000086</v>
+      </c>
+      <c r="E24" s="19">
+        <f>E20-E23</f>
+        <v>-0.35000000000000014</v>
+      </c>
+      <c r="F24" s="19">
+        <f>F20-F23</f>
+        <v>-0.40000000000000241</v>
+      </c>
+      <c r="G24" s="17"/>
+      <c r="H24" s="19"/>
+      <c r="I24" s="19">
+        <f>AVERAGE(D24:F24)</f>
+        <v>-0.4900000000000011</v>
+      </c>
+      <c r="J24" s="17"/>
+    </row>
+    <row r="25" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B25" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="D25" s="29">
+        <f>D21+D23</f>
+        <v>1.01</v>
+      </c>
+      <c r="E25" s="19">
+        <f>E21+E23</f>
+        <v>0.69999999999999973</v>
+      </c>
+      <c r="F25" s="19">
+        <f>F21+F23</f>
+        <v>0.87000000000000122</v>
+      </c>
+      <c r="G25" s="17"/>
+      <c r="H25" s="31">
+        <f>AVERAGE(D25:F25)</f>
+        <v>0.86000000000000032</v>
+      </c>
+      <c r="I25" s="19"/>
+      <c r="J25" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fixje bruto rendement fout MSCI world actiam
</commit_message>
<xml_diff>
--- a/Actiam/Actiam-KostenBepaling2020.xlsx
+++ b/Actiam/Actiam-KostenBepaling2020.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GoogleDrive\Financieel\Aandelen\KeuzeWelkIndexFonds\PerFonds\Actiam\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21449A73-3CF6-414A-A6DD-6F9BA867FAF6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09A8CA3B-498C-48C2-9132-9CBE0DB7D679}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aannames" sheetId="4" r:id="rId1"/>
@@ -89,7 +89,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B18" authorId="0" shapeId="0" xr:uid="{9B32E177-9E47-4B8A-BA3D-C6E6BC6434F4}">
+    <comment ref="B17" authorId="0" shapeId="0" xr:uid="{9B32E177-9E47-4B8A-BA3D-C6E6BC6434F4}">
       <text>
         <r>
           <rPr>
@@ -119,7 +119,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="39">
   <si>
     <t>Gemiddelde</t>
   </si>
@@ -193,12 +193,6 @@
     <t>Actiam AVIAW</t>
   </si>
   <si>
-    <t>Vs gross -ESG</t>
-  </si>
-  <si>
-    <t>Vs net -ESG</t>
-  </si>
-  <si>
     <t>Actiam AVIAOL</t>
   </si>
   <si>
@@ -236,19 +230,24 @@
   </si>
   <si>
     <t>gemiddeld bruto netto index verschil</t>
+  </si>
+  <si>
+    <t>Als Actiam MSCI world had gevolgt</t>
+  </si>
+  <si>
+    <t>(even een snelle schatting 0,02% transactiekosten, nog echt nazoeken)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="6">
+  <numFmts count="5">
     <numFmt numFmtId="44" formatCode="_ &quot;€&quot;\ * #,##0.00_ ;_ &quot;€&quot;\ * \-#,##0.00_ ;_ &quot;€&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="164" formatCode="_ &quot;€&quot;\ * #,##0_ ;_ &quot;€&quot;\ * \-#,##0_ ;_ &quot;€&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="165" formatCode="0.000%"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="0.000"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
@@ -331,7 +330,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -347,6 +346,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -415,7 +420,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Komma" xfId="3" builtinId="3"/>
@@ -776,7 +781,7 @@
         <v>53732257.130000003</v>
       </c>
       <c r="F2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
@@ -883,7 +888,7 @@
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.25">
@@ -906,7 +911,7 @@
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C5" s="11"/>
       <c r="D5" s="11"/>
@@ -1010,13 +1015,15 @@
         <v>2</v>
       </c>
       <c r="C16" s="7">
-        <f>H8+H13</f>
-        <v>0</v>
+        <f>0.15%+0.02%</f>
+        <v>1.7000000000000001E-3</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E16" s="5"/>
+      <c r="E16" s="5" t="s">
+        <v>38</v>
+      </c>
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
       <c r="H16" s="6"/>
@@ -1025,9 +1032,9 @@
       <c r="B17" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C17" s="4" t="e">
-        <f>'Tracking Difference'!#REF!/100</f>
-        <v>#REF!</v>
+      <c r="C17" s="4">
+        <f>'Tracking Difference'!H12/100</f>
+        <v>2.1750000000000016E-3</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>20</v>
@@ -1041,9 +1048,9 @@
       <c r="B18" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C18" s="4" t="e">
+      <c r="C18" s="4">
         <f>C17-C16</f>
-        <v>#REF!</v>
+        <v>4.7500000000000146E-4</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>20</v>
@@ -1076,8 +1083,8 @@
         <v>1</v>
       </c>
       <c r="C21" s="26">
-        <f>F9+H8</f>
-        <v>0</v>
+        <f>0.08%+0.02%</f>
+        <v>1E-3</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>21</v>
@@ -1092,19 +1099,14 @@
       <c r="B23" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C23" s="26" t="e">
+      <c r="C23" s="26">
         <f>C21+C18</f>
-        <v>#REF!</v>
+        <v>1.4750000000000015E-3</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B24" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C24" s="26" t="e">
-        <f>C21+#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="B24" s="1"/>
+      <c r="C24" s="26"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1114,7 +1116,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F528616F-4365-4E03-AA99-F5C2282C78C2}">
-  <dimension ref="B1:K25"/>
+  <dimension ref="B1:K24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46.85546875" customWidth="1"/>
@@ -1163,7 +1165,7 @@
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="15" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C3" s="28">
         <v>11.39</v>
@@ -1175,7 +1177,7 @@
         <v>-3.58</v>
       </c>
       <c r="F3" s="28">
-        <v>30.67</v>
+        <v>30.76</v>
       </c>
       <c r="G3" s="13"/>
       <c r="H3" s="13"/>
@@ -1183,7 +1185,7 @@
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B4" s="15" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C4" s="13">
         <v>10.73</v>
@@ -1246,18 +1248,18 @@
       </c>
       <c r="F6" s="27">
         <f>F3-F2</f>
-        <v>0.20000000000000284</v>
+        <v>0.2900000000000027</v>
       </c>
       <c r="G6" s="13"/>
       <c r="H6" s="16">
         <f>AVERAGE(C6:F6)</f>
-        <v>0.17750000000000066</v>
+        <v>0.20000000000000062</v>
       </c>
       <c r="I6" s="13"/>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B7" s="15" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C7" s="28">
         <f>C3-C4</f>
@@ -1273,17 +1275,17 @@
       </c>
       <c r="F7" s="28">
         <f t="shared" si="0"/>
-        <v>0.65000000000000213</v>
+        <v>0.74000000000000199</v>
       </c>
       <c r="G7" s="13"/>
       <c r="H7" s="16"/>
       <c r="I7" s="13"/>
       <c r="J7" s="32">
         <f>AVERAGE(C7:F7)</f>
-        <v>0.6075000000000006</v>
+        <v>0.63000000000000056</v>
       </c>
       <c r="K7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
@@ -1298,7 +1300,7 @@
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B9" s="15" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C9" s="28">
         <v>0.03</v>
@@ -1317,21 +1319,23 @@
       <c r="I9" s="13"/>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B10" s="15"/>
+      <c r="B10" s="15" t="s">
+        <v>37</v>
+      </c>
       <c r="C10" s="28">
         <f>C2-C9</f>
         <v>11.280000000000001</v>
       </c>
       <c r="D10" s="28">
-        <f t="shared" ref="D10:F10" si="1">D2-D9</f>
+        <f>D2-D9</f>
         <v>7.7799999999999994</v>
       </c>
       <c r="E10" s="28">
-        <f t="shared" si="1"/>
+        <f>E2-E9</f>
         <v>-3.9</v>
       </c>
       <c r="F10" s="28">
-        <f t="shared" si="1"/>
+        <f>F2-F9</f>
         <v>30.64</v>
       </c>
       <c r="G10" s="13"/>
@@ -1339,104 +1343,120 @@
       <c r="I10" s="13"/>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B11" s="15"/>
-      <c r="C11" s="28"/>
-      <c r="D11" s="28"/>
-      <c r="E11" s="28"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="13"/>
+      <c r="B11" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11">
+        <f>C10-C4</f>
+        <v>0.55000000000000071</v>
+      </c>
+      <c r="D11">
+        <f t="shared" ref="D11:F11" si="1">D10-D4</f>
+        <v>0.26999999999999957</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="1"/>
+        <v>0.21000000000000041</v>
+      </c>
+      <c r="F11">
+        <f t="shared" si="1"/>
+        <v>0.62000000000000099</v>
+      </c>
+      <c r="I11" s="16">
+        <f>AVERAGE(C11:F11)</f>
+        <v>0.41250000000000042</v>
+      </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B12" s="15" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="C12" s="28">
-        <f>C5-C9</f>
-        <v>0.55000000000000004</v>
+        <f>C3-C10</f>
+        <v>0.10999999999999943</v>
       </c>
       <c r="D12" s="28">
-        <f>D5-D9</f>
-        <v>0.26999999999999991</v>
+        <f>D3-D10</f>
+        <v>0.32000000000000028</v>
       </c>
       <c r="E12" s="28">
-        <f>E5-E9</f>
-        <v>0.21000000000000046</v>
+        <f>E3-E10</f>
+        <v>0.31999999999999984</v>
       </c>
       <c r="F12" s="28">
-        <f>F5-F9</f>
-        <v>0.61999999999999933</v>
+        <f>F3-F10</f>
+        <v>0.12000000000000099</v>
       </c>
       <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="16">
+      <c r="H12" s="33">
         <f>AVERAGE(C12:F12)</f>
-        <v>0.41249999999999998</v>
-      </c>
+        <v>0.21750000000000014</v>
+      </c>
+      <c r="I12" s="13"/>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B13" s="15" t="s">
+      <c r="B13" s="15"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="16"/>
+    </row>
+    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B15" s="30" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B16" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="28">
-        <f>C6+C9</f>
-        <v>0.11000000000000007</v>
-      </c>
-      <c r="D13" s="28">
-        <f>D6+D9</f>
-        <v>0.31999999999999995</v>
-      </c>
-      <c r="E13" s="28">
-        <f>E6+E9</f>
-        <v>0.31999999999999978</v>
-      </c>
-      <c r="F13" s="28">
-        <f>F6+F9</f>
-        <v>3.000000000000283E-2</v>
-      </c>
-      <c r="G13" s="13"/>
-      <c r="H13" s="33">
-        <f>AVERAGE(C13:F13)</f>
-        <v>0.19500000000000065</v>
-      </c>
-      <c r="I13" s="13"/>
-    </row>
-    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B16" s="30" t="s">
-        <v>31</v>
-      </c>
+      <c r="D16" s="29">
+        <v>8.02</v>
+      </c>
+      <c r="E16" s="19">
+        <v>-10.92</v>
+      </c>
+      <c r="F16" s="17">
+        <v>20.13</v>
+      </c>
+      <c r="G16" s="17"/>
+      <c r="H16" s="17"/>
+      <c r="I16" s="19"/>
+      <c r="J16" s="17"/>
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B17" s="18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D17" s="29">
-        <v>8.02</v>
+        <v>8.6</v>
       </c>
       <c r="E17" s="19">
-        <v>-10.92</v>
+        <v>-9.91</v>
       </c>
       <c r="F17" s="17">
-        <v>20.13</v>
+        <v>21.07</v>
       </c>
       <c r="G17" s="17"/>
-      <c r="H17" s="17"/>
+      <c r="H17" s="19"/>
       <c r="I17" s="19"/>
       <c r="J17" s="17"/>
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B18" s="18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D18" s="29">
-        <v>8.6</v>
+        <v>8.31</v>
       </c>
       <c r="E18" s="19">
-        <v>-9.91</v>
+        <v>-10.26</v>
       </c>
       <c r="F18" s="17">
-        <v>21.07</v>
+        <v>20.6</v>
       </c>
       <c r="G18" s="17"/>
       <c r="H18" s="19"/>
@@ -1444,146 +1464,128 @@
       <c r="J18" s="17"/>
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B19" s="18" t="s">
-        <v>28</v>
+      <c r="B19" s="15" t="s">
+        <v>9</v>
       </c>
       <c r="D19" s="29">
-        <v>8.31</v>
+        <f>D16-D18</f>
+        <v>-0.29000000000000092</v>
       </c>
       <c r="E19" s="19">
-        <v>-10.26</v>
-      </c>
-      <c r="F19" s="17">
-        <v>20.6</v>
-      </c>
-      <c r="G19" s="17"/>
+        <f>E16-E18</f>
+        <v>-0.66000000000000014</v>
+      </c>
+      <c r="F19" s="19">
+        <f>F16-F18</f>
+        <v>-0.47000000000000242</v>
+      </c>
+      <c r="G19" s="19"/>
       <c r="H19" s="19"/>
-      <c r="I19" s="19"/>
+      <c r="I19" s="19">
+        <f>AVERAGE(D19:F19)</f>
+        <v>-0.47333333333333449</v>
+      </c>
       <c r="J19" s="17"/>
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B20" s="15" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D20" s="29">
-        <f>D17-D19</f>
-        <v>-0.29000000000000092</v>
+        <f>D17-D16</f>
+        <v>0.58000000000000007</v>
       </c>
       <c r="E20" s="19">
-        <f>E17-E19</f>
-        <v>-0.66000000000000014</v>
+        <f>E17-E16</f>
+        <v>1.0099999999999998</v>
       </c>
       <c r="F20" s="19">
-        <f>F17-F19</f>
-        <v>-0.47000000000000242</v>
+        <f>F17-F16</f>
+        <v>0.94000000000000128</v>
       </c>
       <c r="G20" s="19"/>
-      <c r="H20" s="19"/>
-      <c r="I20" s="19">
+      <c r="H20" s="19">
         <f>AVERAGE(D20:F20)</f>
-        <v>-0.47333333333333449</v>
-      </c>
+        <v>0.84333333333333371</v>
+      </c>
+      <c r="I20" s="19"/>
       <c r="J20" s="17"/>
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B21" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="D21" s="29">
-        <f>D18-D17</f>
-        <v>0.58000000000000007</v>
-      </c>
-      <c r="E21" s="19">
-        <f>E18-E17</f>
-        <v>1.0099999999999998</v>
-      </c>
-      <c r="F21" s="19">
-        <f>F18-F17</f>
-        <v>0.94000000000000128</v>
-      </c>
+      <c r="B21" s="18"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="19"/>
       <c r="G21" s="19"/>
-      <c r="H21" s="19">
-        <f>AVERAGE(D21:F21)</f>
-        <v>0.84333333333333371</v>
-      </c>
+      <c r="H21" s="19"/>
       <c r="I21" s="19"/>
       <c r="J21" s="17"/>
     </row>
     <row r="22" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B22" s="18"/>
-      <c r="D22" s="29"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="19"/>
-      <c r="G22" s="19"/>
-      <c r="H22" s="19"/>
+      <c r="B22" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="D22" s="29">
+        <v>0.43</v>
+      </c>
+      <c r="E22" s="19">
+        <v>-0.31</v>
+      </c>
+      <c r="F22" s="17">
+        <v>-7.0000000000000007E-2</v>
+      </c>
+      <c r="G22" s="17"/>
+      <c r="H22" s="17"/>
       <c r="I22" s="19"/>
-      <c r="J22" s="17"/>
+      <c r="J22" s="19"/>
     </row>
     <row r="23" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B23" s="15" t="s">
-        <v>36</v>
+      <c r="B23" s="18" t="s">
+        <v>28</v>
       </c>
       <c r="D23" s="29">
-        <v>0.43</v>
+        <f>D19-D22</f>
+        <v>-0.72000000000000086</v>
       </c>
       <c r="E23" s="19">
-        <v>-0.31</v>
-      </c>
-      <c r="F23" s="17">
-        <v>-7.0000000000000007E-2</v>
+        <f>E19-E22</f>
+        <v>-0.35000000000000014</v>
+      </c>
+      <c r="F23" s="19">
+        <f>F19-F22</f>
+        <v>-0.40000000000000241</v>
       </c>
       <c r="G23" s="17"/>
-      <c r="H23" s="17"/>
-      <c r="I23" s="19"/>
-      <c r="J23" s="19"/>
+      <c r="H23" s="19"/>
+      <c r="I23" s="19">
+        <f>AVERAGE(D23:F23)</f>
+        <v>-0.4900000000000011</v>
+      </c>
+      <c r="J23" s="17"/>
     </row>
     <row r="24" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B24" s="18" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D24" s="29">
-        <f>D20-D23</f>
-        <v>-0.72000000000000086</v>
+        <f>D20+D22</f>
+        <v>1.01</v>
       </c>
       <c r="E24" s="19">
-        <f>E20-E23</f>
-        <v>-0.35000000000000014</v>
+        <f>E20+E22</f>
+        <v>0.69999999999999973</v>
       </c>
       <c r="F24" s="19">
-        <f>F20-F23</f>
-        <v>-0.40000000000000241</v>
+        <f>F20+F22</f>
+        <v>0.87000000000000122</v>
       </c>
       <c r="G24" s="17"/>
-      <c r="H24" s="19"/>
-      <c r="I24" s="19">
+      <c r="H24" s="31">
         <f>AVERAGE(D24:F24)</f>
-        <v>-0.4900000000000011</v>
-      </c>
+        <v>0.86000000000000032</v>
+      </c>
+      <c r="I24" s="19"/>
       <c r="J24" s="17"/>
-    </row>
-    <row r="25" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B25" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="D25" s="29">
-        <f>D21+D23</f>
-        <v>1.01</v>
-      </c>
-      <c r="E25" s="19">
-        <f>E21+E23</f>
-        <v>0.69999999999999973</v>
-      </c>
-      <c r="F25" s="19">
-        <f>F21+F23</f>
-        <v>0.87000000000000122</v>
-      </c>
-      <c r="G25" s="17"/>
-      <c r="H25" s="31">
-        <f>AVERAGE(D25:F25)</f>
-        <v>0.86000000000000032</v>
-      </c>
-      <c r="I25" s="19"/>
-      <c r="J25" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>